<commit_message>
fatura, İrsaliye,Talep,Sipariş  sayfalarında css değişiklikleri yapıldı
</commit_message>
<xml_diff>
--- a/WebApplication11/Tema/excel/ornek-cari-listesi.xlsx
+++ b/WebApplication11/Tema/excel/ornek-cari-listesi.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kackinmuharrem\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\YKYonetimPaneli\WebApplication11\Tema\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051CAD65-6B46-4697-A008-291BA7047C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986404FE-7B86-48E5-87C9-986445CFAD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -169,9 +169,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -468,9 +470,9 @@
     <col min="11" max="11" width="8" customWidth="1"/>
     <col min="12" max="12" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.42578125" customWidth="1"/>
-    <col min="15" max="15" width="16" customWidth="1"/>
-    <col min="16" max="16" width="12.140625" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" style="3" customWidth="1"/>
+    <col min="15" max="15" width="16" style="3" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" style="3" customWidth="1"/>
     <col min="17" max="17" width="15.140625" customWidth="1"/>
     <col min="18" max="18" width="13.140625" customWidth="1"/>
     <col min="19" max="19" width="6.7109375" customWidth="1"/>
@@ -530,13 +532,13 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">

</xml_diff>